<commit_message>
Preciser les exemples et trancher les cas limites de la grille
</commit_message>
<xml_diff>
--- a/analyses/m3/grille_classification_cas_G.xlsx
+++ b/analyses/m3/grille_classification_cas_G.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" r:id="R18754e2de0b64f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="2" r:id="Rfbd4771278994688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" r:id="Rd1f6b4878f354480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="2" r:id="Rfa7c5732f5534055"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -252,18 +252,12 @@
     <x:t xml:space="preserve">Classer 8 produits réels</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Une ligne par produit. Listes déroulantes en E, G, H, I. « (à vérifier) » = information à confirmer sur la notice ou le certificat du fabricant.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">N°</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Produit</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Exemple réel à chercher</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Où chercher</x:t>
   </x:si>
   <x:si>
@@ -291,70 +285,46 @@
     <x:t xml:space="preserve">Application ECG d'une montre connectée</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">App ECG de l'Apple Watch (Apple)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Page d'aide Apple « app ECG », notice de l'app</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Tensiomètre connecté (bras)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Withings BPM Connect, ou un tensiomètre Omron connecté</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Fiche produit, notice PDF (logo CE + numéro à 4 chiffres)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Application de méditation et de sommeil</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Petit BamBou (ou Calm, Headspace)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Site de l'éditeur, fiche App Store / Google Play</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Balance connectée « multifonction »</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Withings Body Scan 2 (juin 2026, 500 €) ; à comparer avec Withings BodyFit (juillet 2026)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Fiche produit Withings, notice, FAQ « dispositif médical »</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pompe à insuline patch</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Omnipod (Insulet) ; rappel de lots de pods par l'ANSM le 3 juin 2026</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Site Omnipod, notice, avis de l'ANSM</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Logiciel de télésurveillance cardiaque</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Implicity (inscrit le 20 mai 2026 sur la liste des télésurveillances remboursées) ; comparer avec LATITUDE CLARITY (3 mars 2026)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Site Implicity, avis de la HAS (IMPLICITY IM009)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Détecteur de chute / téléassistance pour personne âgée (cas limite)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Détection des chutes d'une montre connectée ; offre de téléassistance avec détecteur de chute (ex. Présence Verte ou l'offre de votre département)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Site de l'offre, conditions générales, notice du détecteur</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pilulier connecté avec rappels (cas limite)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Medissimo imedipac (pilulier connecté français)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Site Medissimo ; avis de la HAS sur MEDIPAC (21 juin 2022)</x:t>
@@ -930,43 +900,43 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="A2" s="7" t="str">
+        <x:v>Un exemple précis par ligne. « — » = non applicable. Les classes probables et les régimes anciens sont précisés en J. Sources dans les notes des cellules F.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
       <x:c r="A4" s="8" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="s">
+      <x:c r="C4" s="8" t="str">
+        <x:v>Exemple étudié</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="s">
+      <x:c r="E4" s="8" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="s">
+      <x:c r="F4" s="8" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="s">
+      <x:c r="G4" s="8" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="s">
+      <x:c r="H4" s="8" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="s">
+      <x:c r="I4" s="8" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="s">
+      <x:c r="J4" s="8" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="I4" s="8" t="s">
+      <x:c r="K4" s="8" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="J4" s="8" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="K4" s="8" t="s">
-        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="110" customHeight="1">
@@ -974,13 +944,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="9" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="s">
-        <x:v>34</x:v>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>App ECG de l’Apple Watch (Apple), version 2.0 UE</x:v>
       </x:c>
       <x:c r="D5" s="9" t="s">
-        <x:v>35</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
         <x:v>Dispositif médical</x:v>
@@ -998,7 +968,7 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
-        <x:v>L'app analyse le rythme à visée médicale. IIa probable pour l'usage ECG ponctuel décrit, hors surveillance d'urgence (classe/version UE à vérifier). Le périmètre médical ne couvre pas toute la montre.</x:v>
+        <x:v>L’app repère des signes de fibrillation auriculaire. IIa est la proposition du TP pour l’usage décrit, à confirmer sur le certificat UE exact. La montre entière n’est pas un DM. Une aide au diagnostic à risque plus élevé peut relever de IIb ou III.</x:v>
       </x:c>
       <x:c r="K5" s="11" t="str">
         <x:f>IF(E5="","",IF(AND(E5="Bien-être",G5&lt;&gt;"—",G5&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E5="Dispositif médical",OR(G5="—",G5="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G5="IIa",G5="IIb",G5="III"),I5="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G5="I",I5="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F5="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
@@ -1010,19 +980,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="9" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="s">
-        <x:v>37</x:v>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>Withings BPM Connect</x:v>
       </x:c>
       <x:c r="D6" s="9" t="s">
-        <x:v>38</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
         <x:v>Dispositif médical</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>« c'est un outil de diagnostic de qualité médicale »</x:v>
+        <x:v>« c’est un outil de diagnostic de qualité médicale »</x:v>
       </x:c>
       <x:c r="G6" s="10" t="str">
         <x:v>IIa</x:v>
@@ -1034,7 +1004,7 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
-        <x:v>Appareil actif de mesure de la pression artérielle à domicile : IIa, sans surveillance critique immédiate. La classe IIa de la gamme BPM est confirmée par Withings.</x:v>
+        <x:v>Le brassard mesure la pression artérielle pour le suivi de l’hypertension. Appareil actif de mesure : règle 10, classe IIa, organisme notifié requis. Le Bluetooth ne détermine pas la classe.</x:v>
       </x:c>
       <x:c r="K6" s="11" t="str">
         <x:f>IF(E6="","",IF(AND(E6="Bien-être",G6&lt;&gt;"—",G6&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E6="Dispositif médical",OR(G6="—",G6="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G6="IIa",G6="IIb",G6="III"),I6="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G6="I",I6="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F6="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
@@ -1046,13 +1016,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="s">
-        <x:v>40</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>Petit BamBou : application Sommeil</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
-        <x:v>41</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
         <x:v>Bien-être</x:v>
@@ -1070,7 +1040,7 @@
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:v>Finalité de détente et de bien-être, sans diagnostic ni traitement revendiqué d'une maladie. Pas de classe MDR ni d'organisme notifié médical pour cette finalité.</x:v>
+        <x:v>L’éditeur annonce une approche non médicale pour améliorer le sommeil. Conclusion : bien-être. Classe et règle MDR non applicables (—), sans organisme notifié médical. Calm et Headspace ne sont pas les exemples retenus.</x:v>
       </x:c>
       <x:c r="K7" s="11" t="str">
         <x:f>IF(E7="","",IF(AND(E7="Bien-être",G7&lt;&gt;"—",G7&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E7="Dispositif médical",OR(G7="—",G7="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G7="IIa",G7="IIb",G7="III"),I7="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G7="I",I7="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F7="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
@@ -1082,13 +1052,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="9" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="s">
-        <x:v>43</x:v>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="str">
+        <x:v>Withings BodyScan 2 : fonction ECG Monitor 2. Comparaison : BodyFit.</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
-        <x:v>44</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Dispositif médical</x:v>
@@ -1106,7 +1076,7 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:v>IIa probable pour l'analyse ECG, pas pour toutes les fonctions (certificat exact à vérifier). La déclaration ECG App Display concerne un accessoire IIa, règle 3.3. BodyFit : bien-être, sans classe MDR.</x:v>
+        <x:v>La fonction ECG est médicale. IIa/règle 11 reste une proposition pour l’analyse, certificat exact à vérifier. Elle ne classe pas toute la balance. BodyFit est présenté comme non médical. La déclaration ECG App Display concerne un autre module.</x:v>
       </x:c>
       <x:c r="K8" s="11" t="str">
         <x:f>IF(E8="","",IF(AND(E8="Bien-être",G8&lt;&gt;"—",G8&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E8="Dispositif médical",OR(G8="—",G8="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G8="IIa",G8="IIb",G8="III"),I8="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G8="I",I8="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F8="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
@@ -1118,13 +1088,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="9" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="s">
-        <x:v>46</x:v>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="str">
+        <x:v>Omnipod DASH (Insulet)</x:v>
       </x:c>
       <x:c r="D9" s="9" t="s">
-        <x:v>47</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Dispositif médical</x:v>
@@ -1142,25 +1112,25 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:v>Version retenue : DASH. L'administration d'insuline est potentiellement dangereuse en cas d'erreur de débit ou de dose : IIb, cohérent avec l'avis HAS. Ne pas généraliser à toutes les boucles automatisées.</x:v>
+        <x:v>DASH administre de l’insuline. Une erreur de dose ou de débit peut être dangereuse : règle 12, IIb, organisme notifié requis. Ce classement ne s’étend pas automatiquement aux autres versions Omnipod.</x:v>
       </x:c>
       <x:c r="K9" s="11" t="str">
         <x:f>IF(E9="","",IF(AND(E9="Bien-être",G9&lt;&gt;"—",G9&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E9="Dispositif médical",OR(G9="—",G9="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G9="IIa",G9="IIb",G9="III"),I9="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G9="I",I9="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F9="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="130" customHeight="1">
+    <x:row r="10" ht="150" customHeight="1">
       <x:c r="A10" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="9" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C10" s="9" t="s">
-        <x:v>49</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="str">
+        <x:v>Implicity IM009 : classe I déclarée sous la directive 93/42/CEE</x:v>
       </x:c>
       <x:c r="D10" s="9" t="s">
-        <x:v>50</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
         <x:v>Dispositif médical</x:v>
@@ -1170,43 +1140,44 @@
 Traduction : créer des observations cliniquement pertinentes sur l'aggravation de la fibrillation auriculaire.</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>IIa</x:v>
+        <x:v>I</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>Règle 11 (logiciel)</x:v>
+        <x:v>Autre (préciser)</x:v>
       </x:c>
       <x:c r="I10" s="10" t="str">
-        <x:v>Oui</x:v>
+        <x:v>Non</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
-        <x:v>IIa = hypothèse MDR d'aide au suivi différé ; IIb/III si conséquences plus graves (à vérifier). Classe I historique sous directive, en transition selon HAS 2026 : nouvelle classe non établie. Oui vise le scénario MDR IIa.</x:v>
+        <x:v>G et I décrivent la classe I déclarée sous l’ancienne directive et sa procédure initiale sans ON. La règle précise de cette déclaration n’est pas fournie. Sous MDR : règle 11 ; classe actuelle et intervention de l’ON à confirmer. Ne pas présenter IIa comme une certification d’IM009.</x:v>
       </x:c>
       <x:c r="K10" s="11" t="str">
         <x:f>IF(E10="","",IF(AND(E10="Bien-être",G10&lt;&gt;"—",G10&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E10="Dispositif médical",OR(G10="—",G10="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G10="IIa",G10="IIb",G10="III"),I10="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G10="I",I10="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F10="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="225" customHeight="1">
+    <x:row r="11" ht="150" customHeight="1">
       <x:c r="A11" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="9" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="s">
-        <x:v>52</x:v>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="str">
+        <x:v>Apple Watch : fonction Détection des chutes et appel des secours</x:v>
       </x:c>
       <x:c r="D11" s="9" t="s">
-        <x:v>53</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>À discuter</x:v>
+        <x:v>Bien-être</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>Apple : « Si l’Apple Watch détecte une mauvaise chute, elle peut vous mettre en relation avec les services d’urgence. »
-Phrases proposées (fictives) :
-Bien-être : « Alerte un proche en cas de chute pour faciliter l'assistance au quotidien. »
-Médical : « Analyse les troubles de la marche pour aider au diagnostic d'une maladie neurologique. »</x:v>
+Usage retenu : assistance de sécurité.
+Question 4, propositions fictives :
+Bien-être : « Appelle un proche après une chute. »
+Médical : « Analyse la marche pour aider au diagnostic d’une maladie neurologique. »</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
         <x:v>—</x:v>
@@ -1218,34 +1189,35 @@
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>G à I décrivent la seule assistance de sécurité, sans finalité médicale spécifique. L'alternative diagnostique serait un logiciel DM : règle 11, IIa au minimum, ON oui ; niveau exact selon les conséquences (à vérifier).</x:v>
+        <x:v>Position retenue : assistance de sécurité, hors DM pour l’usage décrit. La fonction détecte une chute et appelle les secours, sans diagnostic revendiqué dans la page consultée. Classe/règle MDR non applicables (—), ON médical non requis. « Bien-être » est la catégorie non-DM du modèle.</x:v>
       </x:c>
       <x:c r="K11" s="11" t="str">
         <x:f>IF(E11="","",IF(AND(E11="Bien-être",G11&lt;&gt;"—",G11&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E11="Dispositif médical",OR(G11="—",G11="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G11="IIa",G11="IIb",G11="III"),I11="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G11="I",I11="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F11="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="210" customHeight="1">
+    <x:row r="12" ht="150" customHeight="1">
       <x:c r="A12" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B12" s="9" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="C12" s="9" t="s">
-        <x:v>55</x:v>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C12" s="9" t="str">
+        <x:v>Medissimo imedipac : rappels et suivi des prises (produit historique)</x:v>
       </x:c>
       <x:c r="D12" s="9" t="s">
-        <x:v>56</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
-        <x:v>À discuter</x:v>
+        <x:v>Bien-être</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
-        <x:v>Étude imedipac : « pour assurer l’observance de la délivrance médicamenteuse en temps réel »
-Phrases proposées (fictives) :
-Bien-être : « Rappelle les horaires saisis et signale l'ouverture d'un compartiment. »
-Médical : « Analyse les prises pour recommander au médecin un ajustement personnalisé du traitement. »</x:v>
+        <x:v>Étude imedipac : « pour assurer l’observance de la délivrance médicamenteuse en temps réel ».
+Usage retenu : rappels et traçabilité.
+Question 4, propositions fictives :
+Bien-être : « Rappelle les horaires de prise saisis. »
+Médical : « Analyse les prises pour recommander au médecin un ajustement du traitement. »</x:v>
       </x:c>
       <x:c r="G12" s="10" t="str">
         <x:v>—</x:v>
@@ -1257,14 +1229,14 @@
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>G à I : simple rappel/traçabilité, sans DM. Alternative thérapeutique : règle 11, IIa à III selon risques, ON oui. imedipac retiré en 2018 ; notice à vérifier. HAS 2022 : MEDIPAC non DM selon ANSM, produit distinct.</x:v>
+        <x:v>Position retenue pour les rappels et la traçabilité : organisation des prises, hors DM. Classe/règle MDR non applicables (—), ON médical non requis. L’ouverture d’une case ne prouve pas l’ingestion. imedipac a été retiré en 2018 ; l’avis HAS sur MEDIPAC ne certifie pas ce modèle distinct.</x:v>
       </x:c>
       <x:c r="K12" s="11" t="str">
         <x:f>IF(E12="","",IF(AND(E12="Bien-être",G12&lt;&gt;"—",G12&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E12="Dispositif médical",OR(G12="—",G12="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G12="IIa",G12="IIb",G12="III"),I12="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G12="I",I12="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F12="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="135" customHeight="1">
+    <x:row r="13" ht="145" customHeight="1">
       <x:c r="A13" s="11">
         <x:v>9</x:v>
       </x:c>
@@ -1272,10 +1244,10 @@
         <x:v>Votre projet - cas G : souris ergonomique 1 500 mAh + logiciel</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>Analyse des gestes et recommandations médicales</x:v>
+        <x:v>Cas G : souris ergonomique 1 500 mAh et logiciel de recommandations médicales</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>Finalité proposée à partir du choix de l’équipe ; voir F13 et J13</x:v>
+        <x:v>Finalité proposée pour le TP. Sources réglementaires dans la note F13 et dans le PDF du cas G.</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
         <x:v>Dispositif médical</x:v>
@@ -1293,7 +1265,7 @@
         <x:v>Oui</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>Logiciel d'aide à une décision thérapeutique : IIa probable, sous hypothèse de recommandations non critiques. IIb/III si erreur plus grave. Périmètre souris/logiciel à définir ; 1 500 mAh ne détermine pas la classe.</x:v>
+        <x:v>Le logiciel prévu aide un professionnel à choisir une prise en charge des TMS. IIa probable sous l’hypothèse d’un usage non critique, à confirmer par l’analyse des conséquences d’une erreur. Le prototype n’est pas certifié et son efficacité clinique n’est pas démontrée.</x:v>
       </x:c>
       <x:c r="K13" s="11" t="str">
         <x:f>IF(E13="","",IF(AND(E13="Bien-être",G13&lt;&gt;"—",G13&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E13="Dispositif médical",OR(G13="—",G13="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G13="IIa",G13="IIb",G13="III"),I13="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G13="I",I13="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F13="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
@@ -1302,7 +1274,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="B15" s="12" t="s">
-        <x:v>57</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E15" t="n">
         <x:f>COUNTA(E5:E13)</x:f>
@@ -1311,7 +1283,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="B16" s="12" t="s">
-        <x:v>58</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E16" t="n">
         <x:f>COUNTIF(K5:K13,"OK")</x:f>
@@ -1342,6 +1314,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a23779345144370"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5ee8de59ae84b77"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Completer explicitement les classes et regles non applicables
</commit_message>
<xml_diff>
--- a/analyses/m3/grille_classification_cas_G.xlsx
+++ b/analyses/m3/grille_classification_cas_G.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" r:id="Rd1f6b4878f354480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="2" r:id="Rfa7c5732f5534055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" r:id="R69c4897f934f443d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="2" r:id="R8b4998f0bfea4faa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -901,7 +901,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>Un exemple précis par ligne. « — » = non applicable. Les classes probables et les régimes anciens sont précisés en J. Sources dans les notes des cellules F.</x:v>
+        <x:v>Un exemple précis par ligne. « Non applicable » = usage hors dispositif médical, donc aucune classe ni règle MDR. Classes probables et anciens régimes précisés en J. Sources dans les notes F.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
@@ -971,7 +971,7 @@
         <x:v>L’app repère des signes de fibrillation auriculaire. IIa est la proposition du TP pour l’usage décrit, à confirmer sur le certificat UE exact. La montre entière n’est pas un DM. Une aide au diagnostic à risque plus élevé peut relever de IIb ou III.</x:v>
       </x:c>
       <x:c r="K5" s="11" t="str">
-        <x:f>IF(E5="","",IF(AND(E5="Bien-être",G5&lt;&gt;"—",G5&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E5="Dispositif médical",OR(G5="—",G5="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G5="IIa",G5="IIb",G5="III"),I5="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G5="I",I5="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F5="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E5="","",IF(AND(E5="Bien-être",G5&lt;&gt;"—",G5&lt;&gt;"Non applicable",G5&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E5="Dispositif médical",OR(G5="—",G5="Non applicable",G5="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G5="IIa",G5="IIb",G5="III"),I5="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G5="I",I5="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F5="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1007,7 +1007,7 @@
         <x:v>Le brassard mesure la pression artérielle pour le suivi de l’hypertension. Appareil actif de mesure : règle 10, classe IIa, organisme notifié requis. Le Bluetooth ne détermine pas la classe.</x:v>
       </x:c>
       <x:c r="K6" s="11" t="str">
-        <x:f>IF(E6="","",IF(AND(E6="Bien-être",G6&lt;&gt;"—",G6&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E6="Dispositif médical",OR(G6="—",G6="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G6="IIa",G6="IIb",G6="III"),I6="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G6="I",I6="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F6="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E6="","",IF(AND(E6="Bien-être",G6&lt;&gt;"—",G6&lt;&gt;"Non applicable",G6&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E6="Dispositif médical",OR(G6="—",G6="Non applicable",G6="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G6="IIa",G6="IIb",G6="III"),I6="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G6="I",I6="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F6="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1031,19 +1031,19 @@
         <x:v>« Sommeil avec Petit BamBou propose une approche naturelle et non médicale »</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:v>L’éditeur annonce une approche non médicale pour améliorer le sommeil. Conclusion : bien-être. Classe et règle MDR non applicables (—), sans organisme notifié médical. Calm et Headspace ne sont pas les exemples retenus.</x:v>
+        <x:v>L’éditeur annonce une approche non médicale pour améliorer le sommeil. Conclusion : bien-être. Classe et règle MDR non applicables, sans organisme notifié médical. Calm et Headspace ne sont pas les exemples retenus.</x:v>
       </x:c>
       <x:c r="K7" s="11" t="str">
-        <x:f>IF(E7="","",IF(AND(E7="Bien-être",G7&lt;&gt;"—",G7&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E7="Dispositif médical",OR(G7="—",G7="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G7="IIa",G7="IIb",G7="III"),I7="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G7="I",I7="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F7="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E7="","",IF(AND(E7="Bien-être",G7&lt;&gt;"—",G7&lt;&gt;"Non applicable",G7&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E7="Dispositif médical",OR(G7="—",G7="Non applicable",G7="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G7="IIa",G7="IIb",G7="III"),I7="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G7="I",I7="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F7="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1079,7 +1079,7 @@
         <x:v>La fonction ECG est médicale. IIa/règle 11 reste une proposition pour l’analyse, certificat exact à vérifier. Elle ne classe pas toute la balance. BodyFit est présenté comme non médical. La déclaration ECG App Display concerne un autre module.</x:v>
       </x:c>
       <x:c r="K8" s="11" t="str">
-        <x:f>IF(E8="","",IF(AND(E8="Bien-être",G8&lt;&gt;"—",G8&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E8="Dispositif médical",OR(G8="—",G8="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G8="IIa",G8="IIb",G8="III"),I8="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G8="I",I8="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F8="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E8="","",IF(AND(E8="Bien-être",G8&lt;&gt;"—",G8&lt;&gt;"Non applicable",G8&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E8="Dispositif médical",OR(G8="—",G8="Non applicable",G8="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G8="IIa",G8="IIb",G8="III"),I8="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G8="I",I8="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F8="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1115,7 +1115,7 @@
         <x:v>DASH administre de l’insuline. Une erreur de dose ou de débit peut être dangereuse : règle 12, IIb, organisme notifié requis. Ce classement ne s’étend pas automatiquement aux autres versions Omnipod.</x:v>
       </x:c>
       <x:c r="K9" s="11" t="str">
-        <x:f>IF(E9="","",IF(AND(E9="Bien-être",G9&lt;&gt;"—",G9&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E9="Dispositif médical",OR(G9="—",G9="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G9="IIa",G9="IIb",G9="III"),I9="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G9="I",I9="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F9="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E9="","",IF(AND(E9="Bien-être",G9&lt;&gt;"—",G9&lt;&gt;"Non applicable",G9&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E9="Dispositif médical",OR(G9="—",G9="Non applicable",G9="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G9="IIa",G9="IIb",G9="III"),I9="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G9="I",I9="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F9="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1152,7 +1152,7 @@
         <x:v>G et I décrivent la classe I déclarée sous l’ancienne directive et sa procédure initiale sans ON. La règle précise de cette déclaration n’est pas fournie. Sous MDR : règle 11 ; classe actuelle et intervention de l’ON à confirmer. Ne pas présenter IIa comme une certification d’IM009.</x:v>
       </x:c>
       <x:c r="K10" s="11" t="str">
-        <x:f>IF(E10="","",IF(AND(E10="Bien-être",G10&lt;&gt;"—",G10&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E10="Dispositif médical",OR(G10="—",G10="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G10="IIa",G10="IIb",G10="III"),I10="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G10="I",I10="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F10="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E10="","",IF(AND(E10="Bien-être",G10&lt;&gt;"—",G10&lt;&gt;"Non applicable",G10&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E10="Dispositif médical",OR(G10="—",G10="Non applicable",G10="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G10="IIa",G10="IIb",G10="III"),I10="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G10="I",I10="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F10="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1180,19 +1180,19 @@
 Médical : « Analyse la marche pour aider au diagnostic d’une maladie neurologique. »</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="I11" s="10" t="str">
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>Position retenue : assistance de sécurité, hors DM pour l’usage décrit. La fonction détecte une chute et appelle les secours, sans diagnostic revendiqué dans la page consultée. Classe/règle MDR non applicables (—), ON médical non requis. « Bien-être » est la catégorie non-DM du modèle.</x:v>
+        <x:v>Position retenue : assistance de sécurité, hors DM pour l’usage décrit. La fonction détecte une chute et appelle les secours, sans diagnostic revendiqué dans la page consultée. Classe/règle MDR non applicables, ON médical non requis. « Bien-être » est la catégorie non-DM du modèle.</x:v>
       </x:c>
       <x:c r="K11" s="11" t="str">
-        <x:f>IF(E11="","",IF(AND(E11="Bien-être",G11&lt;&gt;"—",G11&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E11="Dispositif médical",OR(G11="—",G11="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G11="IIa",G11="IIb",G11="III"),I11="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G11="I",I11="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F11="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E11="","",IF(AND(E11="Bien-être",G11&lt;&gt;"—",G11&lt;&gt;"Non applicable",G11&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E11="Dispositif médical",OR(G11="—",G11="Non applicable",G11="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G11="IIa",G11="IIb",G11="III"),I11="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G11="I",I11="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F11="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1220,19 +1220,19 @@
 Médical : « Analyse les prises pour recommander au médecin un ajustement du traitement. »</x:v>
       </x:c>
       <x:c r="G12" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>Non applicable</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
         <x:v>Non</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Position retenue pour les rappels et la traçabilité : organisation des prises, hors DM. Classe/règle MDR non applicables (—), ON médical non requis. L’ouverture d’une case ne prouve pas l’ingestion. imedipac a été retiré en 2018 ; l’avis HAS sur MEDIPAC ne certifie pas ce modèle distinct.</x:v>
+        <x:v>Position retenue pour les rappels et la traçabilité : organisation des prises, hors DM. Classe/règle MDR non applicables, ON médical non requis. L’ouverture d’une case ne prouve pas l’ingestion. imedipac a été retiré en 2018 ; l’avis HAS sur MEDIPAC ne certifie pas ce modèle distinct.</x:v>
       </x:c>
       <x:c r="K12" s="11" t="str">
-        <x:f>IF(E12="","",IF(AND(E12="Bien-être",G12&lt;&gt;"—",G12&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E12="Dispositif médical",OR(G12="—",G12="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G12="IIa",G12="IIb",G12="III"),I12="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G12="I",I12="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F12="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E12="","",IF(AND(E12="Bien-être",G12&lt;&gt;"—",G12&lt;&gt;"Non applicable",G12&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E12="Dispositif médical",OR(G12="—",G12="Non applicable",G12="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G12="IIa",G12="IIb",G12="III"),I12="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G12="I",I12="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F12="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1268,7 +1268,7 @@
         <x:v>Le logiciel prévu aide un professionnel à choisir une prise en charge des TMS. IIa probable sous l’hypothèse d’un usage non critique, à confirmer par l’analyse des conséquences d’une erreur. Le prototype n’est pas certifié et son efficacité clinique n’est pas démontrée.</x:v>
       </x:c>
       <x:c r="K13" s="11" t="str">
-        <x:f>IF(E13="","",IF(AND(E13="Bien-être",G13&lt;&gt;"—",G13&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (—)",IF(AND(E13="Dispositif médical",OR(G13="—",G13="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G13="IIa",G13="IIb",G13="III"),I13="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G13="I",I13="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F13="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
+        <x:f>IF(E13="","",IF(AND(E13="Bien-être",G13&lt;&gt;"—",G13&lt;&gt;"Non applicable",G13&lt;&gt;""),"À revoir : un produit bien-être n'a pas de classe (Non applicable)",IF(AND(E13="Dispositif médical",OR(G13="—",G13="Non applicable",G13="")),"Indiquez une classe : I, IIa, IIb ou III",IF(AND(OR(G13="IIa",G13="IIb",G13="III"),I13="Non"),"À revoir : dès IIa, organisme notifié",IF(AND(G13="I",I13="Oui"),"À vérifier : classe I = en général auto-déclaration",IF(F13="","Ajoutez la phrase qui prouve la finalité","OK"))))))</x:f>
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -1303,17 +1303,17 @@
     <x:dataValidation type="list" allowBlank="1" errorTitle="Valeur non prévue" error="Choisissez une valeur de la liste." promptTitle="Choix" prompt="Bien-être, Dispositif médical ou À discuter" sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13">
       <x:formula1>"Bien-être,Dispositif médical,À discuter"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" errorTitle="Valeur non prévue" error="Choisissez une valeur de la liste." promptTitle="Choix" prompt="I, IIa, IIb, III ou —" sqref="G5 G6 G7 G8 G9 G10 G11 G12 G13">
-      <x:formula1>"I,IIa,IIb,III,—"</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" errorTitle="Valeur non prévue" error="Choisissez une valeur de la liste." promptTitle="Choix" prompt="Oui ou Non" sqref="I5 I6 I7 I8 I9 I10 I11 I12 I13">
       <x:formula1>"Oui,Non"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" errorTitle="Valeur non prévue" error="Choisissez une valeur de la liste." promptTitle="Choix" prompt="Choisissez une règle ou écrivez-la" sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13">
-      <x:formula1>"Règle 11 (logiciel),Règle 10 (appareil de mesure),Règle 12 (administre un médicament),Règle 13 (autre appareil actif),Autre (préciser),—"</x:formula1>
+    <x:dataValidation type="list" sqref="G5:G13">
+      <x:formula1>"I,IIa,IIb,III,—,Non applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H13">
+      <x:formula1>"Règle 11 (logiciel),Règle 10 (appareil de mesure),Règle 12 (administre un médicament),Règle 13 (autre appareil actif),Autre (préciser),—,Non applicable"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5ee8de59ae84b77"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4e3be5b0844fc8"/>
 </x:worksheet>
 </file>
</xml_diff>